<commit_message>
Subindo arquivos da aula 16.03
</commit_message>
<xml_diff>
--- a/OneDrive - SENAC - SP/UC6_Algoritmo/Aula12/cadastro_usuario.xlsx
+++ b/OneDrive - SENAC - SP/UC6_Algoritmo/Aula12/cadastro_usuario.xlsx
@@ -436,16 +436,14 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ds</t>
+          <t>Luis</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>23</t>
-        </is>
+      <c r="B2" t="n">
+        <v>17</v>
       </c>
       <c r="C2" t="n">
-        <v>1.57</v>
+        <v>1.71</v>
       </c>
     </row>
   </sheetData>

</xml_diff>